<commit_message>
Removed the purchase device data read code
</commit_message>
<xml_diff>
--- a/src/test/java/testData/TestData.xlsx
+++ b/src/test/java/testData/TestData.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_Work\Basimane_2026\src\test\java\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF4495B9-2D8F-4B39-A5EF-FA246FF286EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2806C547-0985-4DDB-A183-E8429B8D1851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
   <si>
     <t>Table 1</t>
   </si>
@@ -51,12 +52,48 @@
   <si>
     <t>invalidtest@gmail.com</t>
   </si>
+  <si>
+    <t>DeviceType</t>
+  </si>
+  <si>
+    <t>Apple</t>
+  </si>
+  <si>
+    <t>Phone</t>
+  </si>
+  <si>
+    <t>Colour</t>
+  </si>
+  <si>
+    <t>Blue</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>1 Serengeti Estate</t>
+  </si>
+  <si>
+    <t>Discount</t>
+  </si>
+  <si>
+    <t>SAVE10</t>
+  </si>
+  <si>
+    <t>brand</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="10"/>
       <color indexed="8"/>
@@ -82,6 +119,11 @@
     </font>
     <font>
       <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Helvetica Neue"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color theme="10"/>
       <name val="Helvetica Neue"/>
@@ -113,7 +155,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -300,6 +342,21 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="12"/>
+      </left>
+      <right style="thin">
+        <color indexed="11"/>
+      </right>
+      <top style="thin">
+        <color indexed="12"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyProtection="0">
@@ -309,7 +366,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -353,6 +410,21 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1507,15 +1579,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="27.6" customHeight="1">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="17"/>
-      <c r="F1" s="17"/>
-      <c r="G1" s="18"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="23"/>
     </row>
     <row r="2" spans="1:7" ht="20.25" customHeight="1">
       <c r="A2" s="2" t="s">
@@ -1746,4 +1818,260 @@
     <oddFooter>&amp;C&amp;"Helvetica Neue,Regular"&amp;12&amp;K000000&amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92B2D75D-D9A3-49D8-B038-24AFB9CF3293}">
+  <dimension ref="A1:G23"/>
+  <sheetFormatPr defaultRowHeight="13.2"/>
+  <cols>
+    <col min="1" max="1" width="22.5546875" customWidth="1"/>
+    <col min="2" max="2" width="17.5546875" customWidth="1"/>
+    <col min="3" max="3" width="18.33203125" customWidth="1"/>
+    <col min="4" max="4" width="17.44140625" customWidth="1"/>
+    <col min="5" max="5" width="17.21875" customWidth="1"/>
+    <col min="6" max="6" width="14" customWidth="1"/>
+    <col min="7" max="7" width="17.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="15">
+      <c r="A1" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="21"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="23"/>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="7"/>
+      <c r="D3" s="7"/>
+      <c r="E3" s="7"/>
+      <c r="F3" s="7"/>
+      <c r="G3" s="7"/>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" s="17" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" s="18" t="s">
+        <v>16</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" s="18"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" s="18"/>
+      <c r="B9" s="13"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" s="18"/>
+      <c r="B10" s="13"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" s="18"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="18"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" s="18"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" s="18"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+    </row>
+    <row r="15" spans="1:7">
+      <c r="A15" s="18"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+    </row>
+    <row r="16" spans="1:7">
+      <c r="A16" s="18"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+    </row>
+    <row r="17" spans="1:7">
+      <c r="A17" s="18"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+    </row>
+    <row r="18" spans="1:7">
+      <c r="A18" s="18"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+    </row>
+    <row r="19" spans="1:7">
+      <c r="A19" s="18"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+    </row>
+    <row r="20" spans="1:7">
+      <c r="A20" s="18"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+    </row>
+    <row r="21" spans="1:7">
+      <c r="A21" s="18"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" spans="1:7">
+      <c r="A22" s="18"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+    </row>
+    <row r="23" spans="1:7">
+      <c r="A23" s="19"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Renamed the test data sheet to Login
</commit_message>
<xml_diff>
--- a/src/test/java/testData/TestData.xlsx
+++ b/src/test/java/testData/TestData.xlsx
@@ -8,20 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My_Work\Basimane_2026\src\test\java\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2806C547-0985-4DDB-A183-E8429B8D1851}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23C1631C-09E9-479D-A181-5955965045B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="384" yWindow="384" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Login" sheetId="1" r:id="rId1"/>
+    <sheet name="Purchase" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
     <t>Table 1</t>
   </si>
@@ -53,9 +53,6 @@
     <t>invalidtest@gmail.com</t>
   </si>
   <si>
-    <t>DeviceType</t>
-  </si>
-  <si>
     <t>Apple</t>
   </si>
   <si>
@@ -71,9 +68,6 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t>2</t>
-  </si>
-  <si>
     <t>Address</t>
   </si>
   <si>
@@ -86,7 +80,10 @@
     <t>SAVE10</t>
   </si>
   <si>
-    <t>brand</t>
+    <t>Device</t>
+  </si>
+  <si>
+    <t>Brand</t>
   </si>
 </sst>
 </file>
@@ -125,7 +122,6 @@
     </font>
     <font>
       <sz val="10"/>
-      <color theme="10"/>
       <name val="Helvetica Neue"/>
     </font>
   </fonts>
@@ -366,7 +362,7 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -412,12 +408,6 @@
     <xf numFmtId="49" fontId="4" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="8" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -425,6 +415,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="14" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1579,15 +1572,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="27.6" customHeight="1">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="23"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="22"/>
     </row>
     <row r="2" spans="1:7" ht="20.25" customHeight="1">
       <c r="A2" s="2" t="s">
@@ -1835,49 +1828,61 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="21"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="23"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="22"/>
     </row>
     <row r="2" spans="1:7">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" s="4"/>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-    </row>
-    <row r="3" spans="1:7">
-      <c r="A3" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
+      <c r="C3" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3" s="7">
+        <v>2</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>15</v>
+      </c>
       <c r="G3" s="7"/>
     </row>
     <row r="4" spans="1:7">
-      <c r="A4" s="14" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>11</v>
-      </c>
+      <c r="A4" s="14"/>
+      <c r="B4" s="8"/>
       <c r="C4" s="9"/>
       <c r="D4" s="9"/>
       <c r="E4" s="9"/>
@@ -1885,12 +1890,8 @@
       <c r="G4" s="9"/>
     </row>
     <row r="5" spans="1:7">
-      <c r="A5" s="17" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>13</v>
-      </c>
+      <c r="A5" s="15"/>
+      <c r="B5" s="6"/>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -1898,12 +1899,8 @@
       <c r="G5" s="9"/>
     </row>
     <row r="6" spans="1:7">
-      <c r="A6" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B6" s="11" t="s">
-        <v>15</v>
-      </c>
+      <c r="A6" s="10"/>
+      <c r="B6" s="11"/>
       <c r="C6" s="9"/>
       <c r="D6" s="9"/>
       <c r="E6" s="9"/>
@@ -1911,12 +1908,8 @@
       <c r="G6" s="9"/>
     </row>
     <row r="7" spans="1:7">
-      <c r="A7" s="18" t="s">
-        <v>16</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>17</v>
-      </c>
+      <c r="A7" s="16"/>
+      <c r="B7" s="13"/>
       <c r="C7" s="9"/>
       <c r="D7" s="9"/>
       <c r="E7" s="9"/>
@@ -1924,7 +1917,7 @@
       <c r="G7" s="9"/>
     </row>
     <row r="8" spans="1:7">
-      <c r="A8" s="18"/>
+      <c r="A8" s="16"/>
       <c r="B8" s="13"/>
       <c r="C8" s="9"/>
       <c r="D8" s="9"/>
@@ -1933,7 +1926,7 @@
       <c r="G8" s="9"/>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" s="18"/>
+      <c r="A9" s="16"/>
       <c r="B9" s="13"/>
       <c r="C9" s="9"/>
       <c r="D9" s="9"/>
@@ -1942,7 +1935,7 @@
       <c r="G9" s="9"/>
     </row>
     <row r="10" spans="1:7">
-      <c r="A10" s="18"/>
+      <c r="A10" s="16"/>
       <c r="B10" s="13"/>
       <c r="C10" s="9"/>
       <c r="D10" s="9"/>
@@ -1951,7 +1944,7 @@
       <c r="G10" s="9"/>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="18"/>
+      <c r="A11" s="16"/>
       <c r="B11" s="13"/>
       <c r="C11" s="9"/>
       <c r="D11" s="9"/>
@@ -1960,7 +1953,7 @@
       <c r="G11" s="9"/>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="18"/>
+      <c r="A12" s="16"/>
       <c r="B12" s="13"/>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
@@ -1969,7 +1962,7 @@
       <c r="G12" s="9"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="18"/>
+      <c r="A13" s="16"/>
       <c r="B13" s="13"/>
       <c r="C13" s="9"/>
       <c r="D13" s="9"/>
@@ -1978,7 +1971,7 @@
       <c r="G13" s="9"/>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="18"/>
+      <c r="A14" s="16"/>
       <c r="B14" s="13"/>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
@@ -1987,7 +1980,7 @@
       <c r="G14" s="9"/>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="18"/>
+      <c r="A15" s="16"/>
       <c r="B15" s="13"/>
       <c r="C15" s="9"/>
       <c r="D15" s="9"/>
@@ -1996,7 +1989,7 @@
       <c r="G15" s="9"/>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="18"/>
+      <c r="A16" s="16"/>
       <c r="B16" s="13"/>
       <c r="C16" s="9"/>
       <c r="D16" s="9"/>
@@ -2005,7 +1998,7 @@
       <c r="G16" s="9"/>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="18"/>
+      <c r="A17" s="16"/>
       <c r="B17" s="13"/>
       <c r="C17" s="9"/>
       <c r="D17" s="9"/>
@@ -2014,7 +2007,7 @@
       <c r="G17" s="9"/>
     </row>
     <row r="18" spans="1:7">
-      <c r="A18" s="18"/>
+      <c r="A18" s="16"/>
       <c r="B18" s="13"/>
       <c r="C18" s="9"/>
       <c r="D18" s="9"/>
@@ -2023,7 +2016,7 @@
       <c r="G18" s="9"/>
     </row>
     <row r="19" spans="1:7">
-      <c r="A19" s="18"/>
+      <c r="A19" s="16"/>
       <c r="B19" s="13"/>
       <c r="C19" s="9"/>
       <c r="D19" s="9"/>
@@ -2032,7 +2025,7 @@
       <c r="G19" s="9"/>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="18"/>
+      <c r="A20" s="16"/>
       <c r="B20" s="13"/>
       <c r="C20" s="9"/>
       <c r="D20" s="9"/>
@@ -2041,7 +2034,7 @@
       <c r="G20" s="9"/>
     </row>
     <row r="21" spans="1:7">
-      <c r="A21" s="18"/>
+      <c r="A21" s="16"/>
       <c r="B21" s="13"/>
       <c r="C21" s="9"/>
       <c r="D21" s="9"/>
@@ -2050,7 +2043,7 @@
       <c r="G21" s="9"/>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="18"/>
+      <c r="A22" s="16"/>
       <c r="B22" s="13"/>
       <c r="C22" s="9"/>
       <c r="D22" s="9"/>
@@ -2059,7 +2052,7 @@
       <c r="G22" s="9"/>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="19"/>
+      <c r="A23" s="17"/>
       <c r="B23" s="13"/>
       <c r="C23" s="9"/>
       <c r="D23" s="9"/>

</xml_diff>